<commit_message>
Power_orbit_solar_power_model_1.1.8: final orbit in the sheet (625 km, i 97.5 deg, LTAN 06:00), constellation.m for the 9 satellites, panel area 0.1977 m^2 as a sheet input, ground stations in a Stations sheet, contactTimes.m for downlink windows to the millisecond, downlinkTimes.m for downlink start and end times in seconds, RUN.m for every output in one go, scenarioDemo shows the constellation with the stations, ground tracks optional
</commit_message>
<xml_diff>
--- a/ODIN-Model/assumptions.xlsx
+++ b/ODIN-Model/assumptions.xlsx
@@ -3,13 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" tabRatio="500" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" tabRatio="500" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stations" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Assumptions'!$A$4:$G$29</definedName>
@@ -1510,7 +1511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -1704,7 +1705,7 @@
       <c r="D12" s="19" t="inlineStr"/>
       <c r="E12" s="19" t="inlineStr">
         <is>
-          <t>1/298.257223563. Used only for the drag height.</t>
+          <t>1/298.257223563. Used for the drag height, the ground station positions and the ground track.</t>
         </is>
       </c>
     </row>
@@ -1775,14 +1776,18 @@
         </is>
       </c>
       <c r="C16" s="28" t="n">
-        <v>800</v>
+        <v>625</v>
       </c>
       <c r="D16" s="19" t="inlineStr">
         <is>
           <t>km</t>
         </is>
       </c>
-      <c r="E16" s="19" t="inlineStr"/>
+      <c r="E16" s="19" t="inlineStr">
+        <is>
+          <t>Osculating at the start, orbit-mean altitude about 620.2 km.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="19" t="inlineStr">
@@ -1796,14 +1801,18 @@
         </is>
       </c>
       <c r="C17" s="28" t="n">
-        <v>98.6</v>
+        <v>97.5</v>
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
           <t>deg</t>
         </is>
       </c>
-      <c r="E17" s="19" t="inlineStr"/>
+      <c r="E17" s="19" t="inlineStr">
+        <is>
+          <t>GNC value. Sun synchronous at 625 km would be 97.851 (ssoInclination), so the LTAN drifts about -64 min per year.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="19" t="inlineStr">
@@ -1817,14 +1826,18 @@
         </is>
       </c>
       <c r="C18" s="28" t="n">
-        <v>0</v>
+        <v>83.9718</v>
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
           <t>deg</t>
         </is>
       </c>
-      <c r="E18" s="19" t="inlineStr"/>
+      <c r="E18" s="19" t="inlineStr">
+        <is>
+          <t>LTAN 06:00 at cfg.epoch, mean Sun as in tradeLighting.m. GNC gave 115, which is LTAN 06:00 on 16 Oct 2026.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="19" t="inlineStr">
@@ -1888,23 +1901,23 @@
     <row r="22">
       <c r="A22" s="18" t="inlineStr">
         <is>
-          <t>Switches</t>
+          <t>Constellation</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="19" t="inlineStr">
         <is>
-          <t>J2 acceleration</t>
+          <t>Number of orbit planes</t>
         </is>
       </c>
       <c r="B23" s="19" t="inlineStr">
         <is>
-          <t>cfg.use.J2</t>
-        </is>
-      </c>
-      <c r="C23" s="28" t="b">
-        <v>1</v>
+          <t>cfg.const.nPlanes</t>
+        </is>
+      </c>
+      <c r="C23" s="28" t="n">
+        <v>3</v>
       </c>
       <c r="D23" s="19" t="inlineStr"/>
       <c r="E23" s="19" t="inlineStr"/>
@@ -1912,304 +1925,427 @@
     <row r="24">
       <c r="A24" s="19" t="inlineStr">
         <is>
-          <t>Sun direction and Earth shadow history</t>
+          <t>Satellites per plane</t>
         </is>
       </c>
       <c r="B24" s="19" t="inlineStr">
         <is>
-          <t>cfg.use.eclipse</t>
-        </is>
-      </c>
-      <c r="C24" s="28" t="b">
-        <v>1</v>
+          <t>cfg.const.nPerPlane</t>
+        </is>
+      </c>
+      <c r="C24" s="28" t="n">
+        <v>3</v>
       </c>
       <c r="D24" s="19" t="inlineStr"/>
-      <c r="E24" s="19" t="inlineStr">
-        <is>
-          <t>Needed by solarFlux.m and eclipseTimes.m.</t>
-        </is>
-      </c>
+      <c r="E24" s="19" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="19" t="inlineStr">
         <is>
-          <t>Atmospheric drag in the Jacchia 1977 atmosphere</t>
+          <t>RAAN step between planes</t>
         </is>
       </c>
       <c r="B25" s="19" t="inlineStr">
         <is>
-          <t>cfg.use.drag</t>
-        </is>
-      </c>
-      <c r="C25" s="28" t="b">
-        <v>0</v>
-      </c>
-      <c r="D25" s="19" t="inlineStr"/>
+          <t>cfg.const.dRaan</t>
+        </is>
+      </c>
+      <c r="C25" s="28" t="n">
+        <v>5</v>
+      </c>
+      <c r="D25" s="19" t="inlineStr">
+        <is>
+          <t>deg</t>
+        </is>
+      </c>
       <c r="E25" s="19" t="inlineStr">
         <is>
-          <t>Off by default so existing results are unchanged; set true to include drag.</t>
+          <t>Plane k has RAAN cfg.raan0 + (k-1)*dRaan.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="19" t="inlineStr">
         <is>
-          <t>Solar radiation pressure</t>
+          <t>Along-track step between satellites in a plane</t>
         </is>
       </c>
       <c r="B26" s="19" t="inlineStr">
         <is>
-          <t>cfg.use.srp</t>
-        </is>
-      </c>
-      <c r="C26" s="28" t="b">
-        <v>0</v>
-      </c>
-      <c r="D26" s="19" t="inlineStr"/>
+          <t>cfg.const.dU</t>
+        </is>
+      </c>
+      <c r="C26" s="28" t="n">
+        <v>120</v>
+      </c>
+      <c r="D26" s="19" t="inlineStr">
+        <is>
+          <t>deg</t>
+        </is>
+      </c>
       <c r="E26" s="19" t="inlineStr">
         <is>
-          <t>Not implemented.</t>
+          <t>Taken in time as dU/360 of the nodal period, so a plane shares one trajectory.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="19" t="inlineStr">
-        <is>
-          <t>Shadow geometry</t>
-        </is>
-      </c>
-      <c r="B27" s="19" t="inlineStr">
-        <is>
-          <t>cfg.eclipse.model</t>
-        </is>
-      </c>
-      <c r="C27" s="27" t="inlineStr">
-        <is>
-          <t>conical</t>
-        </is>
-      </c>
-      <c r="D27" s="19" t="inlineStr"/>
-      <c r="E27" s="19" t="inlineStr">
-        <is>
-          <t>'conical' or 'cylindrical'.</t>
+      <c r="A27" s="18" t="inlineStr">
+        <is>
+          <t>Switches</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="18" t="inlineStr">
-        <is>
-          <t>Spacecraft and drag</t>
-        </is>
-      </c>
+      <c r="A28" s="19" t="inlineStr">
+        <is>
+          <t>J2 acceleration</t>
+        </is>
+      </c>
+      <c r="B28" s="19" t="inlineStr">
+        <is>
+          <t>cfg.use.J2</t>
+        </is>
+      </c>
+      <c r="C28" s="28" t="b">
+        <v>1</v>
+      </c>
+      <c r="D28" s="19" t="inlineStr"/>
+      <c r="E28" s="19" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="19" t="inlineStr">
         <is>
-          <t>Spacecraft mass</t>
+          <t>Sun direction and Earth shadow history</t>
         </is>
       </c>
       <c r="B29" s="19" t="inlineStr">
         <is>
-          <t>cfg.drag.mass</t>
-        </is>
-      </c>
-      <c r="C29" s="28" t="n">
-        <v>12</v>
-      </c>
-      <c r="D29" s="19" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
+          <t>cfg.use.eclipse</t>
+        </is>
+      </c>
+      <c r="C29" s="28" t="b">
+        <v>1</v>
+      </c>
+      <c r="D29" s="19" t="inlineStr"/>
       <c r="E29" s="19" t="inlineStr">
         <is>
-          <t>Placeholder</t>
+          <t>Needed by solarFlux.m and eclipseTimes.m.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="19" t="inlineStr">
         <is>
-          <t>Mean cross-sectional area normal to the flow</t>
+          <t>Atmospheric drag in the Jacchia 1977 atmosphere</t>
         </is>
       </c>
       <c r="B30" s="19" t="inlineStr">
         <is>
-          <t>cfg.drag.area</t>
-        </is>
-      </c>
-      <c r="C30" s="28" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="D30" s="19" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
+          <t>cfg.use.drag</t>
+        </is>
+      </c>
+      <c r="C30" s="28" t="b">
+        <v>0</v>
+      </c>
+      <c r="D30" s="19" t="inlineStr"/>
       <c r="E30" s="19" t="inlineStr">
         <is>
-          <t>Placeholder</t>
+          <t>Off by default so existing results are unchanged; set true to include drag.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="19" t="inlineStr">
         <is>
-          <t>Drag coefficient</t>
+          <t>Solar radiation pressure</t>
         </is>
       </c>
       <c r="B31" s="19" t="inlineStr">
         <is>
-          <t>cfg.drag.Cd</t>
-        </is>
-      </c>
-      <c r="C31" s="28" t="n">
-        <v>2.2</v>
+          <t>cfg.use.srp</t>
+        </is>
+      </c>
+      <c r="C31" s="28" t="b">
+        <v>0</v>
       </c>
       <c r="D31" s="19" t="inlineStr"/>
       <c r="E31" s="19" t="inlineStr">
         <is>
-          <t>Placeholder</t>
+          <t>Not implemented.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="19" t="inlineStr">
         <is>
-          <t>10.7 cm solar flux, daily and 81-day mean</t>
+          <t>Shadow geometry</t>
         </is>
       </c>
       <c r="B32" s="19" t="inlineStr">
         <is>
-          <t>cfg.drag.F107</t>
-        </is>
-      </c>
-      <c r="C32" s="28" t="n">
-        <v>150</v>
-      </c>
-      <c r="D32" s="19" t="inlineStr">
-        <is>
-          <t>sfu</t>
-        </is>
-      </c>
+          <t>cfg.eclipse.model</t>
+        </is>
+      </c>
+      <c r="C32" s="27" t="inlineStr">
+        <is>
+          <t>conical</t>
+        </is>
+      </c>
+      <c r="D32" s="19" t="inlineStr"/>
       <c r="E32" s="19" t="inlineStr">
         <is>
-          <t>Held constant for the whole run. CelesTrak forecast mean for Sep 2026 to Sep 2027 is about 107.</t>
+          <t>'conical' or 'cylindrical'.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="18" t="inlineStr">
         <is>
-          <t>Solver</t>
+          <t>Spacecraft and drag</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="19" t="inlineStr">
         <is>
-          <t>ode45 relative error tolerance</t>
+          <t>Spacecraft mass</t>
         </is>
       </c>
       <c r="B34" s="19" t="inlineStr">
         <is>
-          <t>cfg.ode.relTol</t>
-        </is>
-      </c>
-      <c r="C34" s="29" t="n">
-        <v>1e-11</v>
-      </c>
-      <c r="D34" s="19" t="inlineStr"/>
-      <c r="E34" s="19" t="inlineStr"/>
+          <t>cfg.drag.mass</t>
+        </is>
+      </c>
+      <c r="C34" s="28" t="n">
+        <v>12</v>
+      </c>
+      <c r="D34" s="19" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
+      <c r="E34" s="19" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="19" t="inlineStr">
         <is>
-          <t>ode45 absolute error tolerance</t>
+          <t>Mean cross-sectional area normal to the flow</t>
         </is>
       </c>
       <c r="B35" s="19" t="inlineStr">
         <is>
-          <t>cfg.ode.absTol</t>
-        </is>
-      </c>
-      <c r="C35" s="29" t="n">
-        <v>1e-11</v>
-      </c>
-      <c r="D35" s="19" t="inlineStr"/>
-      <c r="E35" s="19" t="inlineStr"/>
+          <t>cfg.drag.area</t>
+        </is>
+      </c>
+      <c r="C35" s="28" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="D35" s="19" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E35" s="19" t="inlineStr">
+        <is>
+          <t>Placeholder</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="19" t="inlineStr">
         <is>
-          <t>Spacing of the uniform output time grid</t>
+          <t>Drag coefficient</t>
         </is>
       </c>
       <c r="B36" s="19" t="inlineStr">
         <is>
-          <t>cfg.ode.dtOut</t>
+          <t>cfg.drag.Cd</t>
         </is>
       </c>
       <c r="C36" s="28" t="n">
-        <v>60</v>
-      </c>
-      <c r="D36" s="19" t="inlineStr">
-        <is>
-          <t>s</t>
-        </is>
-      </c>
+        <v>2.2</v>
+      </c>
+      <c r="D36" s="19" t="inlineStr"/>
       <c r="E36" s="19" t="inlineStr">
         <is>
-          <t>Sets the sampling only, not the integration accuracy.</t>
+          <t>Placeholder</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="18" t="inlineStr">
-        <is>
-          <t>Derived</t>
+      <c r="A37" s="19" t="inlineStr">
+        <is>
+          <t>10.7 cm solar flux, daily and 81-day mean</t>
+        </is>
+      </c>
+      <c r="B37" s="19" t="inlineStr">
+        <is>
+          <t>cfg.drag.F107</t>
+        </is>
+      </c>
+      <c r="C37" s="28" t="n">
+        <v>150</v>
+      </c>
+      <c r="D37" s="19" t="inlineStr">
+        <is>
+          <t>sfu</t>
+        </is>
+      </c>
+      <c r="E37" s="19" t="inlineStr">
+        <is>
+          <t>Held constant for the whole run. CelesTrak forecast mean for Sep 2026 to Sep 2027 is about 107.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="19" t="inlineStr">
-        <is>
-          <t>Ballistic coefficient m/(Cd A)</t>
-        </is>
-      </c>
-      <c r="B38" s="19" t="n"/>
-      <c r="C38" s="30">
-        <f>C29/(C31*C30)</f>
-        <v/>
-      </c>
-      <c r="D38" s="19" t="inlineStr">
-        <is>
-          <t>kg/m²</t>
-        </is>
-      </c>
-      <c r="E38" s="19" t="inlineStr">
-        <is>
-          <t>Derived</t>
+      <c r="A38" s="18" t="inlineStr">
+        <is>
+          <t>Power</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="19" t="inlineStr">
         <is>
+          <t>Solar panel front-face area</t>
+        </is>
+      </c>
+      <c r="B39" s="19" t="inlineStr">
+        <is>
+          <t>cfg.power.panelArea</t>
+        </is>
+      </c>
+      <c r="C39" s="28" t="n">
+        <v>0.1977</v>
+      </c>
+      <c r="D39" s="19" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E39" s="19" t="inlineStr">
+        <is>
+          <t>Total physical area per satellite, passed to arrayPower by main_demo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="18" t="inlineStr">
+        <is>
+          <t>Solver</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="19" t="inlineStr">
+        <is>
+          <t>ode45 relative error tolerance</t>
+        </is>
+      </c>
+      <c r="B41" s="19" t="inlineStr">
+        <is>
+          <t>cfg.ode.relTol</t>
+        </is>
+      </c>
+      <c r="C41" s="29" t="n">
+        <v>1e-11</v>
+      </c>
+      <c r="D41" s="19" t="inlineStr"/>
+      <c r="E41" s="19" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="19" t="inlineStr">
+        <is>
+          <t>ode45 absolute error tolerance</t>
+        </is>
+      </c>
+      <c r="B42" s="19" t="inlineStr">
+        <is>
+          <t>cfg.ode.absTol</t>
+        </is>
+      </c>
+      <c r="C42" s="29" t="n">
+        <v>1e-11</v>
+      </c>
+      <c r="D42" s="19" t="inlineStr"/>
+      <c r="E42" s="19" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="19" t="inlineStr">
+        <is>
+          <t>Spacing of the uniform output time grid</t>
+        </is>
+      </c>
+      <c r="B43" s="19" t="inlineStr">
+        <is>
+          <t>cfg.ode.dtOut</t>
+        </is>
+      </c>
+      <c r="C43" s="28" t="n">
+        <v>60</v>
+      </c>
+      <c r="D43" s="19" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
+      </c>
+      <c r="E43" s="19" t="inlineStr">
+        <is>
+          <t>Sets the sampling only, not the integration accuracy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="18" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="19" t="inlineStr">
+        <is>
+          <t>Ballistic coefficient m/(Cd A)</t>
+        </is>
+      </c>
+      <c r="B45" s="19" t="n"/>
+      <c r="C45" s="30">
+        <f>C34/(C36*C35)</f>
+        <v/>
+      </c>
+      <c r="D45" s="19" t="inlineStr">
+        <is>
+          <t>kg/m²</t>
+        </is>
+      </c>
+      <c r="E45" s="19" t="inlineStr">
+        <is>
+          <t>Derived</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="19" t="inlineStr">
+        <is>
           <t>Exospheric temperature, J77 eq. 20 at Kp = 0</t>
         </is>
       </c>
-      <c r="B39" s="19" t="n"/>
-      <c r="C39" s="30">
-        <f>5.48*C32^0.8+101.8*C32^0.4</f>
+      <c r="B46" s="19" t="n"/>
+      <c r="C46" s="30">
+        <f>5.48*C37^0.8+101.8*C37^0.4</f>
         <v/>
       </c>
-      <c r="D39" s="19" t="inlineStr">
+      <c r="D46" s="19" t="inlineStr">
         <is>
           <t>K</t>
         </is>
       </c>
-      <c r="E39" s="19" t="inlineStr">
+      <c r="E46" s="19" t="inlineStr">
         <is>
           <t>Derived</t>
         </is>
@@ -2222,6 +2358,128 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>Ground stations read by stations.m</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>Latitude [deg]</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>Longitude [deg, east positive]</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="inlineStr">
+        <is>
+          <t>Altitude [m]</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
+        <is>
+          <t>Mask angle [deg]</t>
+        </is>
+      </c>
+      <c r="F4" s="17" t="inlineStr">
+        <is>
+          <t>Use</t>
+        </is>
+      </c>
+      <c r="G4" s="17" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>KSAT Svalbard</t>
+        </is>
+      </c>
+      <c r="B5" s="28" t="n">
+        <v>78.229</v>
+      </c>
+      <c r="C5" s="28" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="D5" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="28" t="n">
+        <v>10</v>
+      </c>
+      <c r="F5" s="28" t="b">
+        <v>1</v>
+      </c>
+      <c r="G5" s="19" t="inlineStr">
+        <is>
+          <t>From the team ground station list, which gives no altitude or mask, so 0 m and 10 deg are assumed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>NASA McMurdo</t>
+        </is>
+      </c>
+      <c r="B6" s="28" t="n">
+        <v>-77.85</v>
+      </c>
+      <c r="C6" s="28" t="n">
+        <v>166.63</v>
+      </c>
+      <c r="D6" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="28" t="n">
+        <v>10</v>
+      </c>
+      <c r="F6" s="28" t="b">
+        <v>1</v>
+      </c>
+      <c r="G6" s="19" t="inlineStr">
+        <is>
+          <t>From the team ground station list, which gives no altitude or mask, so 0 m and 10 deg are assumed.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3119,7 +3377,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>